<commit_message>
Restrict Suggested: Operations Intern to ACT-003 only and add interactive Add Task modal with assignee selector
</commit_message>
<xml_diff>
--- a/EDXSO_Operations_Tracker.xlsx
+++ b/EDXSO_Operations_Tracker.xlsx
@@ -572,7 +572,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Unassigned (Suggested: Operations Intern to draft, Founders to review)</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Unassigned (Suggested: Operations Intern)</t>
+          <t>Unassigned (Requested by Founder 1)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Unassigned (Suggested: Operations Intern)</t>
+          <t>Unassigned</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Standardize role title to Founder's Office Intern across all deliverables, tracker, and drafts
</commit_message>
<xml_diff>
--- a/EDXSO_Operations_Tracker.xlsx
+++ b/EDXSO_Operations_Tracker.xlsx
@@ -619,7 +619,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Unassigned (Suggested: Operations Intern)</t>
+          <t>Unassigned (Suggested: Founder's Office Intern)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -901,7 +901,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Operations Intern</t>
+          <t>Founder's Office Intern</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Confirmed owner is Operations Intern. Central tracker active and maintained weekly.</t>
+          <t>Confirmed owner is Founder's Office Intern. Central tracker active and maintained weekly.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Operations Intern</t>
+          <t>Founder's Office Intern</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">

</xml_diff>